<commit_message>
Prepare HiReTest v1.0.0 public release
</commit_message>
<xml_diff>
--- a/artifacts/results/Hiretest/analysis_3to4.xlsx
+++ b/artifacts/results/Hiretest/analysis_3to4.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本报告" sheetId="1" r:id="Rf60f996714d746ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Version Report" sheetId="1" r:id="R459b704f24614e2f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1257,7 +1257,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>匿名学生</x:v>
+        <x:v>Anonymous Student</x:v>
       </x:c>
       <x:c r="B1" t="s">
         <x:v>0</x:v>

</xml_diff>